<commit_message>
Fix relay safety and add guessing form setup
Bind bot readiness to the current Telegram account, align roster formulas, and preserve complete Unicode content with truthful delivery feedback.

Add alphabetical guessing-form setup and refresh, harden release privacy checks, and update the empty workbook and reconstruction guide.
</commit_message>
<xml_diff>
--- a/templates/angel-mortal-empty.xlsx
+++ b/templates/angel-mortal-empty.xlsx
@@ -654,58 +654,58 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^\s+|\s+$","")&amp;" ["&amp;REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"\s","")&amp;"]",'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$","")&amp;" ["&amp;IF(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]","")="","row "&amp;ROW('Form Responses 1'!A2:A),REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""))&amp;"]",'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="B2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="C2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!D2:D),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!D2:D),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="D2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(LET(choice,_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),IF(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),"Devil",IF(REGEXMATCH(LOWER(TO_TEXT(choice)),"^angel and mortal"),"Angel",""))),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(LET(choice,FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),"Devil",IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^angel and mortal"),"Angel",""))),""))</x:f>
       </x:c>
       <x:c r="E2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="F2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!K2:K),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!K2:K),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="H2" t="str" cm="1">
-        <x:f t="array" ref="H2">IFERROR(MAP($A$2:$A,$G$2:$G,_xlfn.LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(COUNTIF($A$2:$A,mortal)&lt;&gt;1,"",XLOOKUP(mortal,$A$2:$A,$E$2:$E,"")))))),"")</x:f>
+        <x:f t="array" ref="H2">MAP($A$2:$A,$G$2:$G,LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"",IF(EXACT(mortal,participantKey),"",IFNA(INDEX(FILTER($E$2:$E,EXACT($A$2:$A,mortal)),1),"")))))))</x:f>
       </x:c>
       <x:c r="I2" t="str" cm="1">
-        <x:f t="array" ref="I2">IFERROR(MAP($A$2:$A,$G$2:$G,_xlfn.LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(COUNTIF($A$2:$A,mortal)&lt;&gt;1,"",XLOOKUP(mortal,$A$2:$A,$D$2:$D,"")))))),"")</x:f>
+        <x:f t="array" ref="I2">MAP($A$2:$A,$G$2:$G,LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"",IF(EXACT(mortal,participantKey),"",IFNA(INDEX(FILTER($D$2:$D,EXACT($A$2:$A,mortal)),1),"")))))))</x:f>
       </x:c>
       <x:c r="J2" t="str" cm="1">
-        <x:f t="array" ref="J2">IFERROR(MAP($A$2:$A,$G$2:$G,$E$2:$E,$H$2:$H,$I$2:$I,_xlfn.LAMBDA(participantKey,mortal,giverTolerance,mortalTolerance,role,IF(participantKey="","",IF(mortal="","UNASSIGNED",IF(COUNTIF($A$2:$A,mortal)&lt;&gt;1,"INVALID · MORTAL",IF(mortal=participantKey,"INVALID · SELF",IF(role="Angel","READY · ANGEL",IF(role&lt;&gt;"Devil","INVALID · MORTAL MODE",IF(NOT(REGEXMATCH(TO_TEXT(mortalTolerance),"^[1-5]$")),"INVALID · MORTAL TOLERANCE",IF(NOT(REGEXMATCH(TO_TEXT(giverTolerance),"^[1-5]$")),"CHECK · DEVIL ?→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))&lt;=1,"GOOD · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))=2,"CHECK · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,"MISMATCH · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance)))))))))))),"")</x:f>
+        <x:f t="array" ref="J2">MAP($A$2:$A,$G$2:$G,$E$2:$E,$H$2:$H,$I$2:$I,LAMBDA(participantKey,mortal,giverTolerance,mortalTolerance,role,IF(participantKey="","",IF(mortal="","UNASSIGNED",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"UNASSIGNED",IF(EXACT(mortal,participantKey),"UNASSIGNED",IF(role="Angel","READY · ANGEL",IF(role&lt;&gt;"Devil","UNASSIGNED",IF(NOT(REGEXMATCH(TO_TEXT(mortalTolerance),"^[1-5]$")),"INVALID · MORTAL TOLERANCE",IF(NOT(REGEXMATCH(TO_TEXT(giverTolerance),"^[1-5]$")),"CHECK · DEVIL ?→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))&lt;=1,"GOOD · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))=2,"CHECK · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,"MISMATCH · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance))))))))))))</x:f>
       </x:c>
       <x:c r="K2" t="str" cm="1">
-        <x:f t="array" ref="K2">IFERROR(MAP($A$2:$A,$D$2:$D,_xlfn.LAMBDA(participantKey,mode,IF(participantKey="","",IF(COUNTIFS($G$2:$G,participantKey,$A$2:$A,"&lt;&gt;"&amp;participantKey)&lt;&gt;1,"",INDEX(_xlfn._xlws.FILTER($A$2:$A,$G$2:$G=participantKey,$A$2:$A&lt;&gt;participantKey),1)&amp;" — "&amp;mode)))),"")</x:f>
+        <x:f t="array" ref="K2">MAP($A$2:$A,$D$2:$D,LAMBDA(participantKey,mode,IF(participantKey="","",IF(SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&lt;&gt;1,"",INDEX(FILTER($A$2:$A,EXACT($G$2:$G,participantKey),$A$2:$A&lt;&gt;"",NOT(EXACT($A$2:$A,participantKey))),1)&amp;" — "&amp;mode))))</x:f>
       </x:c>
       <x:c r="L2" t="str" cm="1">
-        <x:f t="array" ref="L2">IFERROR(MAP($A$2:$A,$M$2:$M,_xlfn.LAMBDA(participantKey,issues,IF(participantKey="","",IF(issues="","Ready","Review")))),"")</x:f>
+        <x:f t="array" ref="L2">MAP($A$2:$A,$M$2:$M,LAMBDA(participantKey,issues,IF(participantKey="","",IF(issues="","Ready","Review"))))</x:f>
       </x:c>
       <x:c r="M2" t="str" cm="1">
-        <x:f t="array" ref="M2">IFERROR(MAP($A$2:$A,$G$2:$G,$U$2:$U,_xlfn.LAMBDA(participantKey,mortal,formIssues,IF(participantKey="","",TEXTJOIN("; ",TRUE,formIssues,IF(mortal="","Choose a mortal",""),IF(AND(mortal&lt;&gt;"",COUNTIF($A$2:$A,mortal)&lt;&gt;1),"Selected mortal is not a current participant",""),IF(mortal=participantKey,"A participant cannot be their own mortal",""),IF(AND(mortal&lt;&gt;"",mortal&lt;&gt;participantKey,COUNTIF($A$2:$A,mortal)=1,COUNTIFS($G$2:$G,mortal,$A$2:$A,"&lt;&gt;"&amp;mortal)&gt;1),"Selected mortal is assigned to more than one giver",""),IF(COUNTIFS($G$2:$G,participantKey,$A$2:$A,"&lt;&gt;"&amp;participantKey)&lt;&gt;1,"Appears as a mortal "&amp;COUNTIFS($G$2:$G,participantKey,$A$2:$A,"&lt;&gt;"&amp;participantKey)&amp;" times; expected exactly once",""))))),"")</x:f>
+        <x:f t="array" ref="M2">MAP($A$2:$A,$G$2:$G,$U$2:$U,LAMBDA(participantKey,mortal,formIssues,IF(participantKey="","",TEXTJOIN("; ",TRUE,formIssues,IF(mortal="","Choose a mortal",""),IF(AND(mortal&lt;&gt;"",SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1),"Selected mortal is not a current participant",""),IF(EXACT(mortal,participantKey),"A participant cannot be their own mortal",""),IF(AND(mortal&lt;&gt;"",NOT(EXACT(mortal,participantKey)),SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))=1,SUMPRODUCT(N(EXACT($G$2:$G,mortal)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,mortal))))&gt;1),"Selected mortal is assigned to more than one giver",""),IF(SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&lt;&gt;1,"Appears as a mortal "&amp;SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&amp;" times; expected exactly once","")))))</x:f>
       </x:c>
       <x:c r="N2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"\s",""),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="O2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA("form:template:"&amp;_xlfn._xlws.FILTER(ROW('Form Responses 1'!A2:A),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA("form:template:"&amp;FILTER(ROW('Form Responses 1'!A2:A),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="P2" t="str" cm="1">
-        <x:f t="array" ref="P2">IFERROR(IFNA(MAP(_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!G2:G),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!H2:H),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!I2:I),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!J2:J),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!N2:N),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!O2:O),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn.LAMBDA(year,faculty,interests,requirements,choice,tolerance,roomEntry,boundaries,TEXTJOIN(CHAR(10),TRUE,IF(TEXTJOIN(" · ",TRUE,year,faculty)="","",TEXTJOIN(" · ",TRUE,year,faculty)),IF(interests="","","Interests: "&amp;interests),IF(requirements="","","Special requirements: "&amp;requirements),IF(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),"Mode: Devil and Mortal (welfare and pranks).","Mode: Angel and Mortal (welfare only; no pranks)."),IF(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),IF(tolerance="","","Prank tolerance: "&amp;tolerance&amp;"/5"),""),IF(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),IF(roomEntry="","","Room entry: "&amp;roomEntry),""),IF(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),IF(boundaries="","","Off limits: "&amp;boundaries),"")))),""),"")</x:f>
+        <x:f t="array" ref="P2">IFNA(MAP(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!G2:G),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!H2:H),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!I2:I),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!J2:J),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!N2:N),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!O2:O),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),LAMBDA(year,faculty,interests,requirements,choice,tolerance,roomEntry,boundaries,TEXTJOIN(CHAR(10),TRUE,IF(TEXTJOIN(" · ",TRUE,year,faculty)="","",TEXTJOIN(" · ",TRUE,year,faculty)),IF(interests="","","Interests: "&amp;interests),IF(requirements="","","Special requirements: "&amp;requirements),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),"Mode: Devil and Mortal (welfare and pranks).","Mode: Angel and Mortal (welfare only; no pranks)."),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(tolerance="","","Prank tolerance: "&amp;tolerance&amp;"/5"),""),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(roomEntry="","","Room entry: "&amp;roomEntry),""),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(boundaries="","","Off limits: "&amp;boundaries),"")))),"")</x:f>
       </x:c>
       <x:c r="Q2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER(ROW('Form Responses 1'!A2:A),'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER(ROW('Form Responses 1'!A2:A),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="R2" t="str">
-        <x:f>IFERROR(ARRAYFORMULA(IFNA(_xlfn._xlws.FILTER('Form Responses 1'!A2:A,'Form Responses 1'!A2:A&lt;&gt;""),"")),"")</x:f>
+        <x:f>ARRAYFORMULA(IFNA(FILTER('Form Responses 1'!A2:A,'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
       </x:c>
       <x:c r="U2" t="str" cm="1">
-        <x:f t="array" ref="U2">IFERROR(IFNA(MAP(_xlfn._xlws.FILTER('Form Responses 1'!A2:A,'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!D2:D),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"\s",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!P2:P),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn._xlws.FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!N2:N),"^\s+|\s+$",""),'Form Responses 1'!A2:A&lt;&gt;""),_xlfn.LAMBDA(timestamp,name,room,telegramId,choice,declaration,tolerance,roomEntry,IF(timestamp="","",TEXTJOIN("; ",TRUE,IF(name="","Missing name",""),IF(room="","Missing room",""),IF(NOT(REGEXMATCH(TO_TEXT(telegramId),"^\d{5,20}$")),"Telegram ID must contain 5-20 digits",""),IF(NOT(REGEXMATCH(LOWER(TO_TEXT(choice)),"^(angel|devil) and mortal")),"Unknown Angel/Devil selection",""),IF(declaration="","Declaration not accepted",""),IF(AND(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),NOT(REGEXMATCH(TO_TEXT(tolerance),"^[1-5]$"))),"Devil response needs prank tolerance 1-5",""),IF(AND(REGEXMATCH(LOWER(TO_TEXT(choice)),"^devil and mortal"),roomEntry=""),"Devil response needs room-entry preference",""),IF(AND(telegramId&lt;&gt;"",SUMPRODUCT(N($N$2:$N=telegramId))&gt;1),"Duplicate Telegram ID in form responses",""),IF(AND(name&lt;&gt;"",SUMPRODUCT(N(LOWER($B$2:$B)=LOWER(name)))&gt;1),"Duplicate name in form responses",""))))),""),"")</x:f>
+        <x:f t="array" ref="U2">IFNA(MAP(FILTER('Form Responses 1'!A2:A,'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!C2:C),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!D2:D),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!E2:E),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!G2:G),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!H2:H),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!I2:I),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!J2:J),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!K2:K),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!P2:P),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!N2:N),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!O2:O),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),LAMBDA(timestamp,name,gender,room,handle,telegramId,year,faculty,interests,requirements,genderPreference,choice,declaration,tolerance,roomEntry,boundaries,IF(timestamp="","",TEXTJOIN("; ",TRUE,IF(name="","Missing name",""),IF(gender="","Missing gender",""),IF(room="","Missing room",""),IF(handle="","Missing Telegram handle",""),IF(NOT(REGEXMATCH(TO_TEXT(telegramId),"^\d{5,20}$")),"Telegram ID must contain 5-20 digits",""),IF(year="","Missing year of study",""),IF(faculty="","Missing faculty",""),IF(interests="","Missing interests",""),IF(requirements="","Missing special requirements",""),IF(genderPreference="","Missing gender preference",""),IF(NOT(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^(angel|devil) and mortal")),"Unknown Angel/Devil selection",""),IF(declaration="","Declaration not accepted",""),IF(AND(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),NOT(REGEXMATCH(TO_TEXT(tolerance),"^[1-5]$"))),"Devil response needs prank tolerance 1-5",""),IF(AND(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),roomEntry=""),"Devil response needs room-entry preference",""),IF(AND(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),boundaries=""),"Devil response needs boundaries",""),IF(AND(telegramId&lt;&gt;"",SUMPRODUCT(N(EXACT($N$2:$N,telegramId)))&gt;1),"Duplicate Telegram ID in form responses",""),IF(AND(name&lt;&gt;"",SUMPRODUCT(N(LOWER($B$2:$B)=LOWER(name)))&gt;1),"Duplicate name in form responses",""))))),"")</x:f>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Address release review: stable workbook ranges and runtime guidance
</commit_message>
<xml_diff>
--- a/templates/angel-mortal-empty.xlsx
+++ b/templates/angel-mortal-empty.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses 1" sheetId="1" r:id="R4c8f081e61834979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angel Mortal Roster" sheetId="2" r:id="R99808c5f612c45cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses 1" sheetId="1" r:id="R84237a8fed6b4fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angel Mortal Roster" sheetId="2" r:id="R25b9fd6011b04010"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -180,7 +180,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -191,7 +191,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -202,7 +202,7 @@
         <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -213,7 +213,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -224,7 +224,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -235,7 +235,7 @@
         <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -246,7 +246,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -257,7 +257,7 @@
         <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -653,59 +653,59 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$","")&amp;" ["&amp;IF(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]","")="","row "&amp;ROW('Form Responses 1'!A2:A),REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""))&amp;"]",'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!D2:D),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(LET(choice,FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),"Devil",IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^angel and mortal"),"Angel",""))),""))</x:f>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!K2:K),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="H2" t="str" cm="1">
-        <x:f t="array" ref="H2">MAP($A$2:$A,$G$2:$G,LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"",IF(EXACT(mortal,participantKey),"",IFNA(INDEX(FILTER($E$2:$E,EXACT($A$2:$A,mortal)),1),"")))))))</x:f>
-      </x:c>
-      <x:c r="I2" t="str" cm="1">
-        <x:f t="array" ref="I2">MAP($A$2:$A,$G$2:$G,LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"",IF(EXACT(mortal,participantKey),"",IFNA(INDEX(FILTER($D$2:$D,EXACT($A$2:$A,mortal)),1),"")))))))</x:f>
-      </x:c>
-      <x:c r="J2" t="str" cm="1">
-        <x:f t="array" ref="J2">MAP($A$2:$A,$G$2:$G,$E$2:$E,$H$2:$H,$I$2:$I,LAMBDA(participantKey,mortal,giverTolerance,mortalTolerance,role,IF(participantKey="","",IF(mortal="","UNASSIGNED",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"UNASSIGNED",IF(EXACT(mortal,participantKey),"UNASSIGNED",IF(role="Angel","READY · ANGEL",IF(role&lt;&gt;"Devil","UNASSIGNED",IF(NOT(REGEXMATCH(TO_TEXT(mortalTolerance),"^[1-5]$")),"INVALID · MORTAL TOLERANCE",IF(NOT(REGEXMATCH(TO_TEXT(giverTolerance),"^[1-5]$")),"CHECK · DEVIL ?→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))&lt;=1,"GOOD · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))=2,"CHECK · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,"MISMATCH · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance))))))))))))</x:f>
-      </x:c>
-      <x:c r="K2" t="str" cm="1">
-        <x:f t="array" ref="K2">MAP($A$2:$A,$D$2:$D,LAMBDA(participantKey,mode,IF(participantKey="","",IF(SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&lt;&gt;1,"",INDEX(FILTER($A$2:$A,EXACT($G$2:$G,participantKey),$A$2:$A&lt;&gt;"",NOT(EXACT($A$2:$A,participantKey))),1)&amp;" — "&amp;mode))))</x:f>
-      </x:c>
-      <x:c r="L2" t="str" cm="1">
-        <x:f t="array" ref="L2">MAP($A$2:$A,$M$2:$M,LAMBDA(participantKey,issues,IF(participantKey="","",IF(issues="","Ready","Review"))))</x:f>
-      </x:c>
-      <x:c r="M2" t="str" cm="1">
-        <x:f t="array" ref="M2">MAP($A$2:$A,$G$2:$G,$U$2:$U,LAMBDA(participantKey,mortal,formIssues,IF(participantKey="","",TEXTJOIN("; ",TRUE,formIssues,IF(mortal="","Choose a mortal",""),IF(AND(mortal&lt;&gt;"",SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1),"Selected mortal is not a current participant",""),IF(EXACT(mortal,participantKey),"A participant cannot be their own mortal",""),IF(AND(mortal&lt;&gt;"",NOT(EXACT(mortal,participantKey)),SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))=1,SUMPRODUCT(N(EXACT($G$2:$G,mortal)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,mortal))))&gt;1),"Selected mortal is assigned to more than one giver",""),IF(SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&lt;&gt;1,"Appears as a mortal "&amp;SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&amp;" times; expected exactly once","")))))</x:f>
-      </x:c>
-      <x:c r="N2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="O2" t="str">
-        <x:f>ARRAYFORMULA(IFNA("form:template:"&amp;FILTER(ROW('Form Responses 1'!A2:A),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="P2" t="str" cm="1">
-        <x:f t="array" ref="P2">IFNA(MAP(FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!G2:G),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!H2:H),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!I2:I),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!J2:J),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!N2:N),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!O2:O),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),LAMBDA(year,faculty,interests,requirements,choice,tolerance,roomEntry,boundaries,TEXTJOIN(CHAR(10),TRUE,IF(TEXTJOIN(" · ",TRUE,year,faculty)="","",TEXTJOIN(" · ",TRUE,year,faculty)),IF(interests="","","Interests: "&amp;interests),IF(requirements="","","Special requirements: "&amp;requirements),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),"Mode: Devil and Mortal (welfare and pranks).","Mode: Angel and Mortal (welfare only; no pranks)."),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(tolerance="","","Prank tolerance: "&amp;tolerance&amp;"/5"),""),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(roomEntry="","","Room entry: "&amp;roomEntry),""),IF(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(boundaries="","","Off limits: "&amp;boundaries),"")))),"")</x:f>
-      </x:c>
-      <x:c r="Q2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER(ROW('Form Responses 1'!A2:A),'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="R2" t="str">
-        <x:f>ARRAYFORMULA(IFNA(FILTER('Form Responses 1'!A2:A,'Form Responses 1'!A2:A&lt;&gt;""),""))</x:f>
-      </x:c>
-      <x:c r="U2" t="str" cm="1">
-        <x:f t="array" ref="U2">IFNA(MAP(FILTER('Form Responses 1'!A2:A,'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!B2:B),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!C2:C),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!D2:D),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!E2:E),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!F2:F),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!G2:G),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!H2:H),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!I2:I),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!J2:J),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!K2:K),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!L2:L),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!P2:P),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!M2:M),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!N2:N),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),FILTER(REGEXREPLACE(TO_TEXT('Form Responses 1'!O2:O),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),'Form Responses 1'!A2:A&lt;&gt;""),LAMBDA(timestamp,name,gender,room,handle,telegramId,year,faculty,interests,requirements,genderPreference,choice,declaration,tolerance,roomEntry,boundaries,IF(timestamp="","",TEXTJOIN("; ",TRUE,IF(name="","Missing name",""),IF(gender="","Missing gender",""),IF(room="","Missing room",""),IF(handle="","Missing Telegram handle",""),IF(NOT(REGEXMATCH(TO_TEXT(telegramId),"^\d{5,20}$")),"Telegram ID must contain 5-20 digits",""),IF(year="","Missing year of study",""),IF(faculty="","Missing faculty",""),IF(interests="","Missing interests",""),IF(requirements="","Missing special requirements",""),IF(genderPreference="","Missing gender preference",""),IF(NOT(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^(angel|devil) and mortal")),"Unknown Angel/Devil selection",""),IF(declaration="","Declaration not accepted",""),IF(AND(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),NOT(REGEXMATCH(TO_TEXT(tolerance),"^[1-5]$"))),"Devil response needs prank tolerance 1-5",""),IF(AND(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),roomEntry=""),"Devil response needs room-entry preference",""),IF(AND(REGEXMATCH(REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),boundaries=""),"Devil response needs boundaries",""),IF(AND(telegramId&lt;&gt;"",SUMPRODUCT(N(EXACT($N$2:$N,telegramId)))&gt;1),"Duplicate Telegram ID in form responses",""),IF(AND(name&lt;&gt;"",SUMPRODUCT(N(LOWER($B$2:$B)=LOWER(name)))&gt;1),"Duplicate name in form responses",""))))),"")</x:f>
+      <x:c r="A2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!B2:B")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$","")&amp;" ["&amp;IF(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!F2:F")),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]","")="","row "&amp;ROW(INDIRECT("'Form Responses 1'!A2:A")),_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!F2:F")),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""))&amp;"]",INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="B2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!B2:B")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="C2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!D2:D")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="D2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(LET(choice,_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!L2:L")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),IF(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),"Devil",IF(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^angel and mortal"),"Angel",""))),""))</x:f>
+      </x:c>
+      <x:c r="E2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!M2:M")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="F2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!K2:K")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="H2" cm="1">
+        <x:f t="array" ref="H2">_xlfn.MAP($A$2:$A,$G$2:$G,_xlfn.LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"",IF(EXACT(mortal,participantKey),"",_xlfn.IFNA(INDEX(_xlfn._xlws.FILTER($E$2:$E,EXACT($A$2:$A,mortal)),1),"")))))))</x:f>
+      </x:c>
+      <x:c r="I2" cm="1">
+        <x:f t="array" ref="I2">_xlfn.MAP($A$2:$A,$G$2:$G,_xlfn.LAMBDA(participantKey,mortal,IF(participantKey="","",IF(mortal="","",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"",IF(EXACT(mortal,participantKey),"",_xlfn.IFNA(INDEX(_xlfn._xlws.FILTER($D$2:$D,EXACT($A$2:$A,mortal)),1),"")))))))</x:f>
+      </x:c>
+      <x:c r="J2" cm="1">
+        <x:f t="array" ref="J2">_xlfn.MAP($A$2:$A,$G$2:$G,$E$2:$E,$H$2:$H,$I$2:$I,_xlfn.LAMBDA(participantKey,mortal,giverTolerance,mortalTolerance,role,IF(participantKey="","",IF(mortal="","UNASSIGNED",IF(SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1,"UNASSIGNED",IF(EXACT(mortal,participantKey),"UNASSIGNED",IF(role="Angel","READY · ANGEL",IF(role&lt;&gt;"Devil","UNASSIGNED",IF(NOT(REGEXMATCH(TO_TEXT(mortalTolerance),"^[1-5]$")),"INVALID · MORTAL TOLERANCE",IF(NOT(REGEXMATCH(TO_TEXT(giverTolerance),"^[1-5]$")),"CHECK · DEVIL ?→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))&lt;=1,"GOOD · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,IF(ABS(VALUE(giverTolerance)-VALUE(mortalTolerance))=2,"CHECK · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance,"MISMATCH · DEVIL "&amp;giverTolerance&amp;"→"&amp;mortalTolerance))))))))))))</x:f>
+      </x:c>
+      <x:c r="K2" cm="1">
+        <x:f t="array" ref="K2">_xlfn.MAP($A$2:$A,$D$2:$D,_xlfn.LAMBDA(participantKey,mode,IF(participantKey="","",IF(SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&lt;&gt;1,"",INDEX(_xlfn._xlws.FILTER($A$2:$A,EXACT($G$2:$G,participantKey),$A$2:$A&lt;&gt;"",NOT(EXACT($A$2:$A,participantKey))),1)&amp;" — "&amp;mode))))</x:f>
+      </x:c>
+      <x:c r="L2" cm="1">
+        <x:f t="array" ref="L2">_xlfn.MAP($A$2:$A,$M$2:$M,_xlfn.LAMBDA(participantKey,issues,IF(participantKey="","",IF(issues="","Ready","Review"))))</x:f>
+      </x:c>
+      <x:c r="M2" cm="1">
+        <x:f t="array" ref="M2">_xlfn.MAP($A$2:$A,$G$2:$G,$U$2:$U,_xlfn.LAMBDA(participantKey,mortal,formIssues,IF(participantKey="","",_xlfn.TEXTJOIN("; ",TRUE,formIssues,IF(mortal="","Choose a mortal",""),IF(AND(mortal&lt;&gt;"",SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))&lt;&gt;1),"Selected mortal is not a current participant",""),IF(EXACT(mortal,participantKey),"A participant cannot be their own mortal",""),IF(AND(mortal&lt;&gt;"",NOT(EXACT(mortal,participantKey)),SUMPRODUCT(N(EXACT($A$2:$A,mortal)),N($A$2:$A&lt;&gt;""))=1,SUMPRODUCT(N(EXACT($G$2:$G,mortal)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,mortal))))&gt;1),"Selected mortal is assigned to more than one giver",""),IF(SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&lt;&gt;1,"Appears as a mortal "&amp;SUMPRODUCT(N(EXACT($G$2:$G,participantKey)),N($A$2:$A&lt;&gt;""),N(NOT(EXACT($A$2:$A,participantKey))))&amp;" times; expected exactly once","")))))</x:f>
+      </x:c>
+      <x:c r="N2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!F2:F")),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="O2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA("form:template:"&amp;_xlfn._xlws.FILTER(ROW(INDIRECT("'Form Responses 1'!A2:A")),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="P2" cm="1">
+        <x:f t="array" ref="P2">_xlfn.IFNA(_xlfn.MAP(_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!G2:G")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!H2:H")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!I2:I")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!J2:J")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!L2:L")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!M2:M")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!N2:N")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!O2:O")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn.LAMBDA(year,faculty,interests,requirements,choice,tolerance,roomEntry,boundaries,_xlfn.TEXTJOIN(CHAR(10),TRUE,IF(_xlfn.TEXTJOIN(" · ",TRUE,year,faculty)="","",_xlfn.TEXTJOIN(" · ",TRUE,year,faculty)),IF(interests="","","Interests: "&amp;interests),IF(requirements="","","Special requirements: "&amp;requirements),IF(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),"Mode: Devil and Mortal (welfare and pranks).","Mode: Angel and Mortal (welfare only; no pranks)."),IF(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(tolerance="","","Prank tolerance: "&amp;tolerance&amp;"/5"),""),IF(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(roomEntry="","","Room entry: "&amp;roomEntry),""),IF(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),IF(boundaries="","","Off limits: "&amp;boundaries),"")))),"")</x:f>
+      </x:c>
+      <x:c r="Q2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(ROW(INDIRECT("'Form Responses 1'!A2:A")),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="R2">
+        <x:f>ARRAYFORMULA(_xlfn.IFNA(_xlfn._xlws.FILTER(INDIRECT("'Form Responses 1'!A2:A"),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),""))</x:f>
+      </x:c>
+      <x:c r="U2" cm="1">
+        <x:f t="array" ref="U2">_xlfn.IFNA(_xlfn.MAP(_xlfn._xlws.FILTER(INDIRECT("'Form Responses 1'!A2:A"),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!B2:B")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!C2:C")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!D2:D")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!E2:E")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!F2:F")),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!G2:G")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!H2:H")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!I2:I")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!J2:J")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!K2:K")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!L2:L")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!P2:P")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!M2:M")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!N2:N")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn._xlws.FILTER(_xlfn.REGEXREPLACE(TO_TEXT(INDIRECT("'Form Responses 1'!O2:O")),"^[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+|[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+$",""),INDIRECT("'Form Responses 1'!A2:A")&lt;&gt;""),_xlfn.LAMBDA(timestamp,name,gender,room,handle,telegramId,year,faculty,interests,requirements,genderPreference,choice,declaration,tolerance,roomEntry,boundaries,IF(timestamp="","",_xlfn.TEXTJOIN("; ",TRUE,IF(name="","Missing name",""),IF(gender="","Missing gender",""),IF(room="","Missing room",""),IF(handle="","Missing Telegram handle",""),IF(NOT(REGEXMATCH(TO_TEXT(telegramId),"^\d{5,20}$")),"Telegram ID must contain 5-20 digits",""),IF(year="","Missing year of study",""),IF(faculty="","Missing faculty",""),IF(interests="","Missing interests",""),IF(requirements="","Missing special requirements",""),IF(genderPreference="","Missing gender preference",""),IF(NOT(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^(angel|devil) and mortal")),"Unknown Angel/Devil selection",""),IF(declaration="","Declaration not accepted",""),IF(AND(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),NOT(REGEXMATCH(TO_TEXT(tolerance),"^[1-5]$"))),"Devil response needs prank tolerance 1-5",""),IF(AND(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),roomEntry=""),"Devil response needs room-entry preference",""),IF(AND(REGEXMATCH(_xlfn.REGEXREPLACE(LOWER(TO_TEXT(choice)),"[\x{9}\x{a}\x{b}\x{c}\x{d}\x{20}\x{85}\x{a0}\x{1680}\x{2000}\x{2001}\x{2002}\x{2003}\x{2004}\x{2005}\x{2006}\x{2007}\x{2008}\x{2009}\x{200a}\x{2028}\x{2029}\x{202f}\x{205f}\x{3000}\x{feff}]+"," " ),"^devil and mortal"),boundaries=""),"Devil response needs boundaries",""),IF(AND(telegramId&lt;&gt;"",SUMPRODUCT(N(EXACT($N$2:$N,telegramId)))&gt;1),"Duplicate Telegram ID in form responses",""),IF(AND(name&lt;&gt;"",SUMPRODUCT(N(LOWER($B$2:$B)=LOWER(name)))&gt;1),"Duplicate name in form responses",""))))),"")</x:f>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -745,6 +745,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec22f476169840a2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1386a747dfe4a48"/>
 </x:worksheet>
 </file>
</xml_diff>